<commit_message>
Updated output variables and negative test case validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000501/negative/01/data/unit-test-coreid-CG0216-negative.xlsx
+++ b/rules/CORE-000501/negative/01/data/unit-test-coreid-CG0216-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -62,26 +62,13 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -95,22 +82,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <bgColor/>
       </patternFill>
     </fill>
@@ -146,7 +117,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -155,9 +126,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,7 +468,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
       <c r="B2" s="4" t="str">
@@ -527,10 +495,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Subject Visits</v>
       </c>
     </row>
@@ -543,7 +511,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -566,22 +534,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>sv.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>9</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>SVUPDES</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>UNSCHEDULED LABS</v>
       </c>
     </row>
@@ -599,15 +567,35 @@
         <v>9</v>
       </c>
       <c r="E3" s="2" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>WEEK 3: UNSCHEDULED 01</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="str">
+        <v>sv.xpt</v>
+      </c>
+      <c r="C4" s="4" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D4" s="4">
+        <v>9</v>
+      </c>
+      <c r="E4" s="4" t="str">
         <v>VISITDY</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F4" s="4">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -658,113 +646,113 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Pre-specified</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Visit Day</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Start Date/Time of Visit</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>End Date/Time of Visit</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Study Day of Start of Visit</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Study Day of End of Visit</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="5" t="str">
         <v>Description of Unplanned Visit</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
+      <c r="A3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="B3" s="6" t="str">
+      <c r="B3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="C3" s="6" t="str">
+      <c r="C3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="D3" s="6" t="str">
+      <c r="D3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="6" t="str">
+      <c r="E3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="F3" s="6" t="str">
+      <c r="F3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="G3" s="6" t="str">
+      <c r="G3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="H3" s="6" t="str">
+      <c r="H3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="I3" s="6" t="str">
+      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
-      <c r="J3" s="6" t="str">
+      <c r="J3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="K3" s="6" t="str">
+      <c r="K3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="L3" s="6" t="str">
+      <c r="L3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>8</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>200</v>
       </c>
-      <c r="F4" s="6" t="str">
+      <c r="F4" s="5" t="str">
         <v>2</v>
       </c>
-      <c r="G4" s="6" t="str">
+      <c r="G4" s="5" t="str">
         <v>8</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>10</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>8</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>8</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <v>200</v>
       </c>
     </row>
@@ -807,40 +795,40 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B6" s="8" t="str">
+      <c r="B6" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C6" s="8" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="4">
         <v>2</v>
       </c>
-      <c r="E6" s="8" t="str">
+      <c r="E6" s="4" t="str">
         <v>SCREENING 2</v>
       </c>
-      <c r="F6" s="8" t="str">
+      <c r="F6" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G6" s="8" t="str">
+      <c r="G6" s="4" t="str">
         <v>-3</v>
       </c>
-      <c r="H6" s="8" t="str">
+      <c r="H6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="I6" s="8" t="str">
+      <c r="I6" s="4" t="str">
         <v>2012-11-28</v>
       </c>
-      <c r="J6" s="8">
+      <c r="J6" s="4">
         <v>-2</v>
       </c>
-      <c r="K6" s="8">
+      <c r="K6" s="4">
         <v>-2</v>
       </c>
-      <c r="L6" s="8" t="str">
+      <c r="L6" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -883,40 +871,40 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B8" s="8" t="str">
+      <c r="B8" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C8" s="8" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D8" s="8">
+      <c r="D8" s="4">
         <v>4</v>
       </c>
-      <c r="E8" s="8" t="str">
+      <c r="E8" s="4" t="str">
         <v>WEEK 2</v>
       </c>
-      <c r="F8" s="8" t="str">
+      <c r="F8" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G8" s="8" t="str">
+      <c r="G8" s="4" t="str">
         <v>15</v>
       </c>
-      <c r="H8" s="8" t="str">
+      <c r="H8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="I8" s="8" t="str">
+      <c r="I8" s="4" t="str">
         <v>2012-12-13</v>
       </c>
-      <c r="J8" s="8">
+      <c r="J8" s="4">
         <v>14</v>
       </c>
-      <c r="K8" s="8">
+      <c r="K8" s="4">
         <v>14</v>
       </c>
-      <c r="L8" s="8" t="str">
+      <c r="L8" s="4" t="str">
         <v/>
       </c>
     </row>
@@ -933,13 +921,13 @@
       <c r="D9" s="4" t="str">
         <v>4.1</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="6" t="str">
         <v>WEEK 3: UNSCHEDULED 01</v>
       </c>
       <c r="F9" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G9" s="9" t="str">
+      <c r="G9" s="7" t="str">
         <v>24</v>
       </c>
       <c r="H9" s="4" t="str">
@@ -954,7 +942,7 @@
       <c r="K9" s="4" t="str">
         <v>23</v>
       </c>
-      <c r="L9" s="10" t="str">
+      <c r="L9" s="7" t="str">
         <v>UNSCHEDULED LABS</v>
       </c>
     </row>
@@ -997,40 +985,40 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="str">
+      <c r="A11" s="4" t="str">
         <v>CDISCPILOT01</v>
       </c>
-      <c r="B11" s="8" t="str">
+      <c r="B11" s="4" t="str">
         <v>SV</v>
       </c>
-      <c r="C11" s="8" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D11" s="8" t="str">
+      <c r="D11" s="4" t="str">
         <v>6</v>
       </c>
-      <c r="E11" s="8" t="str">
+      <c r="E11" s="4" t="str">
         <v>WEEK 6</v>
       </c>
-      <c r="F11" s="8" t="str">
+      <c r="F11" s="4" t="str">
         <v>Y</v>
       </c>
-      <c r="G11" s="8" t="str">
+      <c r="G11" s="4" t="str">
         <v>43</v>
       </c>
-      <c r="H11" s="8" t="str">
+      <c r="H11" s="4" t="str">
         <v>2013-01-10</v>
       </c>
-      <c r="I11" s="8" t="str">
+      <c r="I11" s="4" t="str">
         <v>2013-01-10</v>
       </c>
-      <c r="J11" s="8" t="str">
+      <c r="J11" s="4" t="str">
         <v>42</v>
       </c>
-      <c r="K11" s="8" t="str">
+      <c r="K11" s="4" t="str">
         <v>42</v>
       </c>
-      <c r="L11" s="8" t="str">
+      <c r="L11" s="4" t="str">
         <v/>
       </c>
     </row>

</xml_diff>